<commit_message>
feat: pipeline completo — 11 provincias, 110 secciones, 704 figuras
Corrida integra de run_all.R: las 11 provincias x 10 secciones terminan OK en
5,8 minutos. Produce 110 archivos de tablas y 704 figuras (PNG 300 dpi y PDF
vectorial). Revision visual de la provincia 11 (Area Metropolitana, el caso
extremo por incluir Medellin): el sistema visual se sostiene en barras con
resalte, barras agrupadas y dumbbells.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/03_Outputs/Turistica_Agroecologica/02_Demografia/demografia.xlsx
+++ b/03_Outputs/Turistica_Agroecologica/02_Demografia/demografia.xlsx
@@ -680,31 +680,31 @@
         </is>
       </c>
       <c r="E2" s="4">
-        <v>10105</v>
+        <v>11015</v>
       </c>
       <c r="F2" s="10">
-        <v>0.156785775240105</v>
+        <v>0.164914959875434</v>
       </c>
       <c r="G2" s="6">
-        <v>3006</v>
+        <v>2928</v>
       </c>
       <c r="H2" s="12">
-        <v>0.29747649678377</v>
+        <v>0.265819337267363</v>
       </c>
       <c r="I2" s="14">
-        <v>0.125595387315117</v>
+        <v>0.128759894459103</v>
       </c>
       <c r="J2" s="8">
-        <v>7099</v>
+        <v>8087</v>
       </c>
       <c r="K2" s="16">
-        <v>0.70252350321623</v>
+        <v>0.734180662732637</v>
       </c>
       <c r="L2" s="18">
-        <v>0.175210405508799</v>
+        <v>0.183578498138564</v>
       </c>
       <c r="M2" s="20">
-        <v>28.4479398590338</v>
+        <v>31.0098028250626</v>
       </c>
     </row>
     <row r="3">
@@ -727,31 +727,31 @@
         </is>
       </c>
       <c r="E3" s="4">
-        <v>12914</v>
+        <v>12612</v>
       </c>
       <c r="F3" s="10">
-        <v>0.200369272780872</v>
+        <v>0.188825008983112</v>
       </c>
       <c r="G3" s="6">
-        <v>3163</v>
+        <v>2709</v>
       </c>
       <c r="H3" s="12">
-        <v>0.244927985132414</v>
+        <v>0.214795432921028</v>
       </c>
       <c r="I3" s="14">
-        <v>0.132155093172892</v>
+        <v>0.119129287598945</v>
       </c>
       <c r="J3" s="8">
-        <v>9751</v>
+        <v>9903</v>
       </c>
       <c r="K3" s="16">
-        <v>0.755072014867586</v>
+        <v>0.785204567078972</v>
       </c>
       <c r="L3" s="18">
-        <v>0.24066441246884</v>
+        <v>0.22480250612912</v>
       </c>
       <c r="M3" s="20">
-        <v>54.3108496747386</v>
+        <v>53.040764759006</v>
       </c>
     </row>
     <row r="4">
@@ -774,31 +774,31 @@
         </is>
       </c>
       <c r="E4" s="4">
-        <v>5988</v>
+        <v>6404</v>
       </c>
       <c r="F4" s="10">
-        <v>0.0929077904144234</v>
+        <v>0.0958797460773745</v>
       </c>
       <c r="G4" s="6">
-        <v>2567</v>
+        <v>2533</v>
       </c>
       <c r="H4" s="12">
-        <v>0.428690714762859</v>
+        <v>0.395534041224235</v>
       </c>
       <c r="I4" s="14">
-        <v>0.107253279852929</v>
+        <v>0.111389621811785</v>
       </c>
       <c r="J4" s="8">
-        <v>3421</v>
+        <v>3871</v>
       </c>
       <c r="K4" s="16">
-        <v>0.571309285237141</v>
+        <v>0.604465958775765</v>
       </c>
       <c r="L4" s="18">
-        <v>0.0844336944986055</v>
+        <v>0.0878734223190775</v>
       </c>
       <c r="M4" s="20">
-        <v>64.0465886094768</v>
+        <v>68.496051011204</v>
       </c>
     </row>
     <row r="5">
@@ -821,31 +821,31 @@
         </is>
       </c>
       <c r="E5" s="4">
-        <v>5754</v>
+        <v>5038</v>
       </c>
       <c r="F5" s="10">
-        <v>0.0892771252579479</v>
+        <v>0.0754281949934124</v>
       </c>
       <c r="G5" s="6">
-        <v>2813</v>
+        <v>2289</v>
       </c>
       <c r="H5" s="12">
-        <v>0.488877302745916</v>
+        <v>0.454346963080588</v>
       </c>
       <c r="I5" s="14">
-        <v>0.11753154508231</v>
+        <v>0.10065963060686</v>
       </c>
       <c r="J5" s="8">
-        <v>2941</v>
+        <v>2749</v>
       </c>
       <c r="K5" s="16">
-        <v>0.511122697254084</v>
+        <v>0.545653036919412</v>
       </c>
       <c r="L5" s="18">
-        <v>0.0725868154108152</v>
+        <v>0.0624035231090529</v>
       </c>
       <c r="M5" s="20">
-        <v>50.1006418628843</v>
+        <v>43.8663596985073</v>
       </c>
     </row>
     <row r="6">
@@ -868,31 +868,31 @@
         </is>
       </c>
       <c r="E6" s="4">
-        <v>3350</v>
+        <v>3469</v>
       </c>
       <c r="F6" s="10">
-        <v>0.0519774712572342</v>
+        <v>0.0519373577673973</v>
       </c>
       <c r="G6" s="6">
-        <v>434</v>
+        <v>377</v>
       </c>
       <c r="H6" s="12">
-        <v>0.12955223880597</v>
+        <v>0.108676852118766</v>
       </c>
       <c r="I6" s="14">
-        <v>0.0181331996323222</v>
+        <v>0.0165787159190853</v>
       </c>
       <c r="J6" s="8">
-        <v>2916</v>
+        <v>3092</v>
       </c>
       <c r="K6" s="16">
-        <v>0.87044776119403</v>
+        <v>0.891323147881234</v>
       </c>
       <c r="L6" s="18">
-        <v>0.0719697904583261</v>
+        <v>0.0701897757196041</v>
       </c>
       <c r="M6" s="20">
-        <v>38.5118594454623</v>
+        <v>39.8798926615847</v>
       </c>
     </row>
     <row r="7">
@@ -915,31 +915,31 @@
         </is>
       </c>
       <c r="E7" s="4">
-        <v>9731</v>
+        <v>9909</v>
       </c>
       <c r="F7" s="10">
-        <v>0.150982917254969</v>
+        <v>0.148356090549766</v>
       </c>
       <c r="G7" s="6">
-        <v>3792</v>
+        <v>3524</v>
       </c>
       <c r="H7" s="12">
-        <v>0.389682458123523</v>
+        <v>0.355636290241195</v>
       </c>
       <c r="I7" s="14">
-        <v>0.158435698169967</v>
+        <v>0.154969217238347</v>
       </c>
       <c r="J7" s="8">
-        <v>5939</v>
+        <v>6385</v>
       </c>
       <c r="K7" s="16">
-        <v>0.610317541876477</v>
+        <v>0.644363709758805</v>
       </c>
       <c r="L7" s="18">
-        <v>0.146580447713306</v>
+        <v>0.144942340869881</v>
       </c>
       <c r="M7" s="20">
-        <v>36.6151352505188</v>
+        <v>37.2849013664978</v>
       </c>
     </row>
     <row r="8">
@@ -962,31 +962,31 @@
         </is>
       </c>
       <c r="E8" s="4">
-        <v>16609</v>
+        <v>18345</v>
       </c>
       <c r="F8" s="10">
-        <v>0.257699647794448</v>
+        <v>0.274658641753503</v>
       </c>
       <c r="G8" s="6">
-        <v>8159</v>
+        <v>8380</v>
       </c>
       <c r="H8" s="12">
-        <v>0.491239689325065</v>
+        <v>0.456800218043063</v>
       </c>
       <c r="I8" s="14">
-        <v>0.340895796774463</v>
+        <v>0.368513632365875</v>
       </c>
       <c r="J8" s="8">
-        <v>8450</v>
+        <v>9965</v>
       </c>
       <c r="K8" s="16">
-        <v>0.508760310674935</v>
+        <v>0.543199781956937</v>
       </c>
       <c r="L8" s="18">
-        <v>0.208554433941309</v>
+        <v>0.226209933714701</v>
       </c>
       <c r="M8" s="20">
-        <v>102.991510551601</v>
+        <v>113.756352644296</v>
       </c>
     </row>
     <row r="9">
@@ -1011,31 +1011,31 @@
         </is>
       </c>
       <c r="E9" s="5">
-        <v>64451</v>
+        <v>66792</v>
       </c>
       <c r="F9" s="11">
         <v>1</v>
       </c>
       <c r="G9" s="7">
-        <v>23934</v>
+        <v>22740</v>
       </c>
       <c r="H9" s="13">
-        <v>0.37135187972258</v>
+        <v>0.340459935321595</v>
       </c>
       <c r="I9" s="15">
         <v>1</v>
       </c>
       <c r="J9" s="9">
-        <v>40517</v>
+        <v>44052</v>
       </c>
       <c r="K9" s="17">
-        <v>0.62864812027742</v>
+        <v>0.659540064678405</v>
       </c>
       <c r="L9" s="19">
         <v>1</v>
       </c>
       <c r="M9" s="21">
-        <v>48.9991544663757</v>
+        <v>50.778909948925</v>
       </c>
     </row>
     <row r="10">
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="E10" s="5">
-        <v>223750</v>
+        <v>225788</v>
       </c>
       <c r="F10" s="11" t="inlineStr">
         <is>
@@ -1068,10 +1068,10 @@
         </is>
       </c>
       <c r="G10" s="7">
-        <v>94892</v>
+        <v>88348</v>
       </c>
       <c r="H10" s="13">
-        <v>0.424098324022346</v>
+        <v>0.39128740234202</v>
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
@@ -1079,10 +1079,10 @@
         </is>
       </c>
       <c r="J10" s="9">
-        <v>128858</v>
+        <v>137440</v>
       </c>
       <c r="K10" s="17">
-        <v>0.575901675977654</v>
+        <v>0.60871259765798</v>
       </c>
       <c r="L10" s="19" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="M10" s="21">
-        <v>29.6510472855187</v>
+        <v>29.9211202882802</v>
       </c>
     </row>
     <row r="11">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="E11" s="5">
-        <v>6951825</v>
+        <v>6928372</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
@@ -1123,10 +1123,10 @@
         </is>
       </c>
       <c r="G11" s="7">
-        <v>5600952</v>
+        <v>5450720</v>
       </c>
       <c r="H11" s="13">
-        <v>0.80568081043467</v>
+        <v>0.786724500358814</v>
       </c>
       <c r="I11" s="15" t="inlineStr">
         <is>
@@ -1134,10 +1134,10 @@
         </is>
       </c>
       <c r="J11" s="9">
-        <v>1350873</v>
+        <v>1477652</v>
       </c>
       <c r="K11" s="17">
-        <v>0.19431918956533</v>
+        <v>0.213275499641186</v>
       </c>
       <c r="L11" s="19" t="inlineStr">
         <is>
@@ -1145,7 +1145,7 @@
         </is>
       </c>
       <c r="M11" s="21">
-        <v>110.689548218114</v>
+        <v>110.316120812453</v>
       </c>
     </row>
   </sheetData>
@@ -2485,13 +2485,13 @@
         </is>
       </c>
       <c r="E9" s="81">
-        <v>7.15566031110226</v>
+        <v>7.26538912806343</v>
       </c>
       <c r="F9" s="83">
-        <v>4.76078614593952</v>
+        <v>4.68926390282652</v>
       </c>
       <c r="G9" s="85">
-        <v>33.1009217478572</v>
+        <v>32.8147459458113</v>
       </c>
     </row>
     <row r="10">
@@ -2516,13 +2516,13 @@
         </is>
       </c>
       <c r="E10" s="81">
-        <v>8.31899198468538</v>
+        <v>8.34133878260628</v>
       </c>
       <c r="F10" s="83">
-        <v>4.93072146613824</v>
+        <v>4.90402610078376</v>
       </c>
       <c r="G10" s="85">
-        <v>30.3187804389163</v>
+        <v>30.2492370183753</v>
       </c>
     </row>
     <row r="11">
@@ -2547,13 +2547,13 @@
         </is>
       </c>
       <c r="E11" s="81">
-        <v>8.68409340580495</v>
+        <v>8.63819084562529</v>
       </c>
       <c r="F11" s="83">
-        <v>5.66384584790104</v>
+        <v>5.63888092494405</v>
       </c>
       <c r="G11" s="85">
-        <v>32.006905849399</v>
+        <v>32.052654940463</v>
       </c>
     </row>
   </sheetData>
@@ -2839,13 +2839,13 @@
         </is>
       </c>
       <c r="E9" s="87">
-        <v>2.26108199481764</v>
+        <v>2.27146325823735</v>
       </c>
       <c r="F9" s="89">
-        <v>1.48229551776818</v>
+        <v>1.43394799728513</v>
       </c>
       <c r="G9" s="91">
-        <v>3.06093251026727</v>
+        <v>3.12011860158836</v>
       </c>
     </row>
     <row r="10">
@@ -2870,13 +2870,13 @@
         </is>
       </c>
       <c r="E10" s="87">
-        <v>1.3497525234784</v>
+        <v>1.36963640191563</v>
       </c>
       <c r="F10" s="89">
-        <v>0.913896103289903</v>
+        <v>0.910301066336893</v>
       </c>
       <c r="G10" s="91">
-        <v>1.61723823854627</v>
+        <v>1.65713154831215</v>
       </c>
     </row>
     <row r="11">
@@ -2901,13 +2901,13 @@
         </is>
       </c>
       <c r="E11" s="87">
-        <v>2.43831542235291</v>
+        <v>2.43784156596946</v>
       </c>
       <c r="F11" s="89">
-        <v>2.30723350389532</v>
+        <v>2.2991539975123</v>
       </c>
       <c r="G11" s="91">
-        <v>2.84838135541031</v>
+        <v>2.88568680338064</v>
       </c>
     </row>
   </sheetData>
@@ -2951,10 +2951,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>10105</v>
+        <v>11015</v>
       </c>
       <c r="C2">
-        <v>0.156785775240105</v>
+        <v>0.164914959875434</v>
       </c>
     </row>
     <row r="3">
@@ -2964,10 +2964,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>12914</v>
+        <v>12612</v>
       </c>
       <c r="C3">
-        <v>0.200369272780872</v>
+        <v>0.188825008983112</v>
       </c>
     </row>
     <row r="4">
@@ -2977,10 +2977,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>5988</v>
+        <v>6404</v>
       </c>
       <c r="C4">
-        <v>0.0929077904144234</v>
+        <v>0.0958797460773745</v>
       </c>
     </row>
     <row r="5">
@@ -2990,10 +2990,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>5754</v>
+        <v>5038</v>
       </c>
       <c r="C5">
-        <v>0.0892771252579479</v>
+        <v>0.0754281949934124</v>
       </c>
     </row>
     <row r="6">
@@ -3003,10 +3003,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>3350</v>
+        <v>3469</v>
       </c>
       <c r="C6">
-        <v>0.0519774712572342</v>
+        <v>0.0519373577673973</v>
       </c>
     </row>
     <row r="7">
@@ -3016,10 +3016,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>9731</v>
+        <v>9909</v>
       </c>
       <c r="C7">
-        <v>0.150982917254969</v>
+        <v>0.148356090549766</v>
       </c>
     </row>
     <row r="8">
@@ -3029,10 +3029,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>16609</v>
+        <v>18345</v>
       </c>
       <c r="C8">
-        <v>0.257699647794448</v>
+        <v>0.274658641753503</v>
       </c>
     </row>
   </sheetData>
@@ -3088,16 +3088,16 @@
         </is>
       </c>
       <c r="B2">
-        <v>3006</v>
+        <v>2928</v>
       </c>
       <c r="C2">
-        <v>0.29747649678377</v>
+        <v>0.265819337267363</v>
       </c>
       <c r="D2">
-        <v>7099</v>
+        <v>8087</v>
       </c>
       <c r="E2">
-        <v>0.70252350321623</v>
+        <v>0.734180662732637</v>
       </c>
     </row>
     <row r="3">
@@ -3107,16 +3107,16 @@
         </is>
       </c>
       <c r="B3">
-        <v>3163</v>
+        <v>2709</v>
       </c>
       <c r="C3">
-        <v>0.244927985132414</v>
+        <v>0.214795432921028</v>
       </c>
       <c r="D3">
-        <v>9751</v>
+        <v>9903</v>
       </c>
       <c r="E3">
-        <v>0.755072014867586</v>
+        <v>0.785204567078972</v>
       </c>
     </row>
     <row r="4">
@@ -3126,16 +3126,16 @@
         </is>
       </c>
       <c r="B4">
-        <v>2567</v>
+        <v>2533</v>
       </c>
       <c r="C4">
-        <v>0.428690714762859</v>
+        <v>0.395534041224235</v>
       </c>
       <c r="D4">
-        <v>3421</v>
+        <v>3871</v>
       </c>
       <c r="E4">
-        <v>0.571309285237141</v>
+        <v>0.604465958775765</v>
       </c>
     </row>
     <row r="5">
@@ -3145,16 +3145,16 @@
         </is>
       </c>
       <c r="B5">
-        <v>2813</v>
+        <v>2289</v>
       </c>
       <c r="C5">
-        <v>0.488877302745916</v>
+        <v>0.454346963080588</v>
       </c>
       <c r="D5">
-        <v>2941</v>
+        <v>2749</v>
       </c>
       <c r="E5">
-        <v>0.511122697254084</v>
+        <v>0.545653036919412</v>
       </c>
     </row>
     <row r="6">
@@ -3164,16 +3164,16 @@
         </is>
       </c>
       <c r="B6">
-        <v>434</v>
+        <v>377</v>
       </c>
       <c r="C6">
-        <v>0.12955223880597</v>
+        <v>0.108676852118766</v>
       </c>
       <c r="D6">
-        <v>2916</v>
+        <v>3092</v>
       </c>
       <c r="E6">
-        <v>0.87044776119403</v>
+        <v>0.891323147881234</v>
       </c>
     </row>
     <row r="7">
@@ -3183,16 +3183,16 @@
         </is>
       </c>
       <c r="B7">
-        <v>3792</v>
+        <v>3524</v>
       </c>
       <c r="C7">
-        <v>0.389682458123523</v>
+        <v>0.355636290241195</v>
       </c>
       <c r="D7">
-        <v>5939</v>
+        <v>6385</v>
       </c>
       <c r="E7">
-        <v>0.610317541876477</v>
+        <v>0.644363709758805</v>
       </c>
     </row>
     <row r="8">
@@ -3202,16 +3202,16 @@
         </is>
       </c>
       <c r="B8">
-        <v>8159</v>
+        <v>8380</v>
       </c>
       <c r="C8">
-        <v>0.491239689325065</v>
+        <v>0.456800218043063</v>
       </c>
       <c r="D8">
-        <v>8450</v>
+        <v>9965</v>
       </c>
       <c r="E8">
-        <v>0.508760310674935</v>
+        <v>0.543199781956937</v>
       </c>
     </row>
   </sheetData>
@@ -3254,10 +3254,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>10105</v>
+        <v>11015</v>
       </c>
       <c r="C2">
-        <v>28.4479398590338</v>
+        <v>31.0098028250626</v>
       </c>
     </row>
     <row r="3">
@@ -3267,10 +3267,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>12914</v>
+        <v>12612</v>
       </c>
       <c r="C3">
-        <v>54.3108496747386</v>
+        <v>53.040764759006</v>
       </c>
     </row>
     <row r="4">
@@ -3280,10 +3280,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>5988</v>
+        <v>6404</v>
       </c>
       <c r="C4">
-        <v>64.0465886094768</v>
+        <v>68.496051011204</v>
       </c>
     </row>
     <row r="5">
@@ -3293,10 +3293,10 @@
         </is>
       </c>
       <c r="B5">
-        <v>5754</v>
+        <v>5038</v>
       </c>
       <c r="C5">
-        <v>50.1006418628843</v>
+        <v>43.8663596985073</v>
       </c>
     </row>
     <row r="6">
@@ -3306,10 +3306,10 @@
         </is>
       </c>
       <c r="B6">
-        <v>3350</v>
+        <v>3469</v>
       </c>
       <c r="C6">
-        <v>38.5118594454623</v>
+        <v>39.8798926615847</v>
       </c>
     </row>
     <row r="7">
@@ -3319,10 +3319,10 @@
         </is>
       </c>
       <c r="B7">
-        <v>9731</v>
+        <v>9909</v>
       </c>
       <c r="C7">
-        <v>36.6151352505188</v>
+        <v>37.2849013664978</v>
       </c>
     </row>
     <row r="8">
@@ -3332,10 +3332,10 @@
         </is>
       </c>
       <c r="B8">
-        <v>16609</v>
+        <v>18345</v>
       </c>
       <c r="C8">
-        <v>102.991510551601</v>
+        <v>113.756352644296</v>
       </c>
     </row>
   </sheetData>

</xml_diff>